<commit_message>
tanhieu_fix UI and logic be
</commit_message>
<xml_diff>
--- a/EmployeeManagement/App_Data/EmployeeTemplate.xlsx
+++ b/EmployeeManagement/App_Data/EmployeeTemplate.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21240" windowHeight="11445"/>
+    <workbookView windowWidth="28800" windowHeight="11460"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1242,7 +1242,7 @@
   <cols>
     <col min="1" max="1" width="23.4285714285714" customWidth="1"/>
     <col min="2" max="2" width="17.2857142857143" customWidth="1"/>
-    <col min="3" max="3" width="22.4285714285714" customWidth="1"/>
+    <col min="3" max="3" width="28.8571428571429" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
tanhieu_feat: add client and server side validation
</commit_message>
<xml_diff>
--- a/EmployeeManagement/App_Data/EmployeeTemplate.xlsx
+++ b/EmployeeManagement/App_Data/EmployeeTemplate.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>社員一覧表</t>
   </si>
@@ -44,7 +44,10 @@
     <t>部署</t>
   </si>
   <si>
-    <t>生年月日</t>
+    <t>メール</t>
+  </si>
+  <si>
+    <t xml:space="preserve">生年月日 </t>
   </si>
 </sst>
 </file>
@@ -1237,44 +1240,49 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="4" outlineLevelCol="3"/>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="4" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="23.4285714285714" customWidth="1"/>
-    <col min="2" max="2" width="17.2857142857143" customWidth="1"/>
-    <col min="3" max="3" width="28.8571428571429" customWidth="1"/>
-    <col min="4" max="4" width="23" customWidth="1"/>
+    <col min="1" max="1" width="18.4285714285714" customWidth="1"/>
+    <col min="2" max="2" width="27.4285714285714" customWidth="1"/>
+    <col min="3" max="3" width="34.7142857142857" customWidth="1"/>
+    <col min="4" max="4" width="29.5714285714286" customWidth="1"/>
+    <col min="5" max="5" width="26.8571428571429" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" spans="1:4">
+    <row r="1" ht="15.75" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:5">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:5">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:5">
       <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
@@ -1287,11 +1295,14 @@
       <c r="D5" s="3" t="s">
         <v>5</v>
       </c>
+      <c r="E5" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>